<commit_message>
feat: add BraTS 2019 benchmark pipeline, results (10-80%), and 39-paper SSL literature synthesis
</commit_message>
<xml_diff>
--- a/runs/benchmark_master_results.xlsx
+++ b/runs/benchmark_master_results.xlsx
@@ -136,7 +136,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -185,6 +185,9 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -559,11 +562,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M9"/>
+  <dimension ref="A1:M13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="118" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
     <col width="24" customWidth="1" min="3" max="3"/>
     <col width="19" customWidth="1" min="4" max="4"/>
     <col width="42" customWidth="1" min="5" max="5"/>
@@ -886,63 +889,315 @@
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
         <is>
+          <t>ratio_70</t>
+        </is>
+      </c>
+      <c r="B9" s="13" t="inlineStr">
+        <is>
+          <t>70% Labeled (71 Cases)</t>
+        </is>
+      </c>
+      <c r="C9" s="14" t="n">
+        <v>71</v>
+      </c>
+      <c r="D9" s="14" t="n">
+        <v>31</v>
+      </c>
+      <c r="E9" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F9" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G9" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H9" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I9" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J9" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K9" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L9" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M9" s="18" t="inlineStr">
+        <is>
+          <t>In Progress...</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
           <t>ratio_80</t>
         </is>
       </c>
-      <c r="B9" s="13" t="inlineStr">
+      <c r="B10" s="7" t="inlineStr">
         <is>
           <t>80% Labeled (82 Cases)</t>
         </is>
       </c>
-      <c r="C9" s="14" t="n">
+      <c r="C10" s="8" t="n">
         <v>82</v>
       </c>
-      <c r="D9" s="14" t="n">
+      <c r="D10" s="8" t="n">
         <v>20</v>
       </c>
-      <c r="E9" s="15" t="inlineStr">
+      <c r="E10" s="9" t="inlineStr">
         <is>
           <t>75.40%</t>
         </is>
       </c>
-      <c r="F9" s="15" t="inlineStr">
+      <c r="F10" s="9" t="inlineStr">
         <is>
           <t>54.21%</t>
         </is>
       </c>
-      <c r="G9" s="15" t="inlineStr">
+      <c r="G10" s="9" t="inlineStr">
         <is>
           <t>55.45%</t>
         </is>
       </c>
-      <c r="H9" s="16" t="inlineStr">
+      <c r="H10" s="10" t="inlineStr">
         <is>
           <t>61.69%</t>
         </is>
       </c>
-      <c r="I9" s="15" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J9" s="15" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K9" s="15" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L9" s="16" t="inlineStr">
+      <c r="I10" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J10" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K10" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L10" s="10" t="inlineStr">
         <is>
           <t>65.23%</t>
         </is>
       </c>
-      <c r="M9" s="17" t="inlineStr">
+      <c r="M10" s="17" t="inlineStr">
         <is>
           <t>+3.54%</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="12" t="inlineStr">
+        <is>
+          <t>ratio_30</t>
+        </is>
+      </c>
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>30% Labeled (31 Cases)</t>
+        </is>
+      </c>
+      <c r="C11" s="14" t="n">
+        <v>31</v>
+      </c>
+      <c r="D11" s="14" t="n">
+        <v>71</v>
+      </c>
+      <c r="E11" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F11" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G11" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H11" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I11" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J11" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K11" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L11" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M11" s="18" t="inlineStr">
+        <is>
+          <t>In Progress...</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>ratio_50</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>50% Labeled (51 Cases)</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="n">
+        <v>51</v>
+      </c>
+      <c r="D12" s="8" t="n">
+        <v>51</v>
+      </c>
+      <c r="E12" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F12" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G12" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H12" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I12" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J12" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K12" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L12" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M12" s="18" t="inlineStr">
+        <is>
+          <t>In Progress...</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="12" t="inlineStr">
+        <is>
+          <t>ratio_100</t>
+        </is>
+      </c>
+      <c r="B13" s="13" t="inlineStr">
+        <is>
+          <t>100% Labeled (102 Cases)</t>
+        </is>
+      </c>
+      <c r="C13" s="14" t="n">
+        <v>102</v>
+      </c>
+      <c r="D13" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F13" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G13" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H13" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I13" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J13" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K13" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L13" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M13" s="18" t="inlineStr">
+        <is>
+          <t>In Progress...</t>
         </is>
       </c>
     </row>
@@ -1024,28 +1279,28 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="18" t="inlineStr">
+      <c r="A4" s="19" t="inlineStr">
         <is>
           <t>ratio_10</t>
         </is>
       </c>
-      <c r="B4" s="19" t="n">
+      <c r="B4" s="20" t="n">
         <v>10</v>
       </c>
-      <c r="C4" s="19" t="n">
+      <c r="C4" s="20" t="n">
         <v>195</v>
       </c>
-      <c r="D4" s="20" t="inlineStr">
+      <c r="D4" s="21" t="inlineStr">
         <is>
           <t>62.76%</t>
         </is>
       </c>
-      <c r="E4" s="20" t="inlineStr">
+      <c r="E4" s="21" t="inlineStr">
         <is>
           <t>63.04%</t>
         </is>
       </c>
-      <c r="F4" s="20" t="inlineStr">
+      <c r="F4" s="21" t="inlineStr">
         <is>
           <t>65.73%</t>
         </is>
@@ -1057,28 +1312,28 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="18" t="inlineStr">
+      <c r="A5" s="19" t="inlineStr">
         <is>
           <t>ratio_20</t>
         </is>
       </c>
-      <c r="B5" s="19" t="n">
+      <c r="B5" s="20" t="n">
         <v>20</v>
       </c>
-      <c r="C5" s="19" t="n">
+      <c r="C5" s="20" t="n">
         <v>155</v>
       </c>
-      <c r="D5" s="20" t="inlineStr">
+      <c r="D5" s="21" t="inlineStr">
         <is>
           <t>65.91%</t>
         </is>
       </c>
-      <c r="E5" s="20" t="inlineStr">
+      <c r="E5" s="21" t="inlineStr">
         <is>
           <t>64.61%</t>
         </is>
       </c>
-      <c r="F5" s="20" t="inlineStr">
+      <c r="F5" s="21" t="inlineStr">
         <is>
           <t>65.25%</t>
         </is>
@@ -1090,28 +1345,28 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="18" t="inlineStr">
+      <c r="A6" s="19" t="inlineStr">
         <is>
           <t>ratio_40</t>
         </is>
       </c>
-      <c r="B6" s="19" t="n">
+      <c r="B6" s="20" t="n">
         <v>41</v>
       </c>
-      <c r="C6" s="19" t="n">
+      <c r="C6" s="20" t="n">
         <v>95</v>
       </c>
-      <c r="D6" s="20" t="inlineStr">
+      <c r="D6" s="21" t="inlineStr">
         <is>
           <t>69.42%</t>
         </is>
       </c>
-      <c r="E6" s="20" t="inlineStr">
+      <c r="E6" s="21" t="inlineStr">
         <is>
           <t>58.12%</t>
         </is>
       </c>
-      <c r="F6" s="20" t="inlineStr">
+      <c r="F6" s="21" t="inlineStr">
         <is>
           <t>64.50%</t>
         </is>
@@ -1123,28 +1378,28 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="18" t="inlineStr">
+      <c r="A7" s="19" t="inlineStr">
         <is>
           <t>ratio_80</t>
         </is>
       </c>
-      <c r="B7" s="19" t="n">
+      <c r="B7" s="20" t="n">
         <v>82</v>
       </c>
-      <c r="C7" s="19" t="n">
+      <c r="C7" s="20" t="n">
         <v>65</v>
       </c>
-      <c r="D7" s="20" t="inlineStr">
+      <c r="D7" s="21" t="inlineStr">
         <is>
           <t>75.40%</t>
         </is>
       </c>
-      <c r="E7" s="20" t="inlineStr">
+      <c r="E7" s="21" t="inlineStr">
         <is>
           <t>54.21%</t>
         </is>
       </c>
-      <c r="F7" s="20" t="inlineStr">
+      <c r="F7" s="21" t="inlineStr">
         <is>
           <t>55.45%</t>
         </is>

</xml_diff>